<commit_message>
Release v2.3.0 evidence-gated tracking plans
</commit_message>
<xml_diff>
--- a/skill/assets/default-tracking-plan.xlsx
+++ b/skill/assets/default-tracking-plan.xlsx
@@ -628,16 +628,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:B5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="36" customWidth="1" min="4" max="4"/>
-    <col width="40" customWidth="1" min="5" max="5"/>
-    <col width="32" customWidth="1" min="6" max="6"/>
-    <col width="28" customWidth="1" min="7" max="7"/>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="96" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
@@ -657,53 +652,23 @@
     <row r="4" ht="34" customHeight="1">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>Journey</t>
+          <t>Event</t>
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr">
         <is>
-          <t>Event</t>
-        </is>
-      </c>
-      <c r="C4" s="6" t="inlineStr">
-        <is>
-          <t>Classification</t>
-        </is>
-      </c>
-      <c r="D4" s="6" t="inlineStr">
-        <is>
           <t>Definition</t>
-        </is>
-      </c>
-      <c r="E4" s="6" t="inlineStr">
-        <is>
-          <t>Trigger</t>
-        </is>
-      </c>
-      <c r="F4" s="6" t="inlineStr">
-        <is>
-          <t>Pages / routes / components</t>
-        </is>
-      </c>
-      <c r="G4" s="6" t="inlineStr">
-        <is>
-          <t>Event-specific variables</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n"/>
       <c r="B5" s="4" t="n"/>
-      <c r="C5" s="4" t="n"/>
-      <c r="D5" s="4" t="n"/>
-      <c r="E5" s="4" t="n"/>
-      <c r="F5" s="4" t="n"/>
-      <c r="G5" s="4" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="A1:B1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -802,18 +767,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I12"/>
+  <dimension ref="A1:G12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="23" customWidth="1" min="5" max="5"/>
-    <col width="38" customWidth="1" min="6" max="6"/>
-    <col width="36" customWidth="1" min="7" max="7"/>
-    <col width="22" customWidth="1" min="8" max="8"/>
-    <col width="32" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="42" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
@@ -909,27 +872,17 @@
       </c>
       <c r="E11" s="6" t="inlineStr">
         <is>
-          <t>Condition</t>
+          <t>Definition</t>
         </is>
       </c>
       <c r="F11" s="6" t="inlineStr">
         <is>
-          <t>Definition</t>
+          <t>Possible values / rule</t>
         </is>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
-          <t>Possible values / rule</t>
-        </is>
-      </c>
-      <c r="H11" s="6" t="inlineStr">
-        <is>
           <t>Example</t>
-        </is>
-      </c>
-      <c r="I11" s="6" t="inlineStr">
-        <is>
-          <t>dataLayer path / source</t>
         </is>
       </c>
     </row>
@@ -941,20 +894,18 @@
       <c r="E12" s="4" t="n"/>
       <c r="F12" s="4" t="n"/>
       <c r="G12" s="4" t="n"/>
-      <c r="H12" s="4" t="n"/>
-      <c r="I12" s="4" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="9">
-    <mergeCell ref="B9:I9"/>
-    <mergeCell ref="A2:I2"/>
-    <mergeCell ref="B7:I7"/>
-    <mergeCell ref="B6:I6"/>
-    <mergeCell ref="A1:I1"/>
-    <mergeCell ref="B3:I3"/>
-    <mergeCell ref="B5:I5"/>
-    <mergeCell ref="B8:I8"/>
-    <mergeCell ref="B4:I4"/>
+    <mergeCell ref="B3:G3"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="B5:G5"/>
+    <mergeCell ref="B9:G9"/>
+    <mergeCell ref="B8:G8"/>
+    <mergeCell ref="B4:G4"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="B7:G7"/>
+    <mergeCell ref="B6:G6"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Release v2.5.0 variant-aware tracking plans
</commit_message>
<xml_diff>
--- a/skill/assets/default-tracking-plan.xlsx
+++ b/skill/assets/default-tracking-plan.xlsx
@@ -680,16 +680,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
     <col width="11" customWidth="1" min="2" max="2"/>
     <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="38" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="38" customWidth="1" min="6" max="6"/>
-    <col width="28" customWidth="1" min="7" max="7"/>
+    <col width="42" customWidth="1" min="4" max="4"/>
+    <col width="42" customWidth="1" min="5" max="5"/>
+    <col width="32" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
@@ -729,17 +728,12 @@
       </c>
       <c r="E4" s="6" t="inlineStr">
         <is>
-          <t>Example</t>
+          <t>Rule</t>
         </is>
       </c>
       <c r="F4" s="6" t="inlineStr">
         <is>
-          <t>Possible values / rule</t>
-        </is>
-      </c>
-      <c r="G4" s="6" t="inlineStr">
-        <is>
-          <t>Concerned events</t>
+          <t>Possible values or examples</t>
         </is>
       </c>
     </row>
@@ -750,12 +744,11 @@
       <c r="D5" s="4" t="n"/>
       <c r="E5" s="4" t="n"/>
       <c r="F5" s="4" t="n"/>
-      <c r="G5" s="4" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A1:F1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -801,7 +794,7 @@
       </c>
       <c r="B3" s="4" t="n"/>
     </row>
-    <row r="4" ht="32" customHeight="1">
+    <row r="4" hidden="1" ht="32" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Classification</t>
@@ -877,12 +870,12 @@
       </c>
       <c r="F11" s="6" t="inlineStr">
         <is>
-          <t>Possible values / rule</t>
+          <t>Rule</t>
         </is>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
-          <t>Example</t>
+          <t>Possible values or examples</t>
         </is>
       </c>
     </row>

</xml_diff>